<commit_message>
Update: atur 1 file absensi per hari
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi April 22 2026 Wednesday 10_27_21.xlsx
+++ b/PC-06/docs/Absensi April 22 2026 Wednesday 10_27_21.xlsx
@@ -1109,8 +1109,16 @@
       <c r="U7" s="8" t="n"/>
       <c r="V7" s="8" t="n"/>
       <c r="W7" s="8" t="n"/>
-      <c r="X7" s="8" t="n"/>
-      <c r="Y7" s="8" t="n"/>
+      <c r="X7" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="Y7" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Z7" s="8" t="n"/>
       <c r="AA7" s="8" t="n"/>
       <c r="AB7" s="8" t="n"/>
@@ -1387,7 +1395,11 @@
       <c r="U12" s="8" t="n"/>
       <c r="V12" s="8" t="n"/>
       <c r="W12" s="8" t="n"/>
-      <c r="X12" s="8" t="n"/>
+      <c r="X12" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="Y12" s="8" t="n"/>
       <c r="Z12" s="8" t="n"/>
       <c r="AA12" s="8" t="n"/>
@@ -1687,7 +1699,11 @@
         </is>
       </c>
       <c r="T17" s="8" t="n"/>
-      <c r="U17" s="8" t="n"/>
+      <c r="U17" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="V17" s="8" t="n"/>
       <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>

</xml_diff>

<commit_message>
Add: absensi trigger file
</commit_message>
<xml_diff>
--- a/PC-06/docs/Absensi April 22 2026 Wednesday 10_27_21.xlsx
+++ b/PC-06/docs/Absensi April 22 2026 Wednesday 10_27_21.xlsx
@@ -6097,8 +6097,16 @@
       <c r="AC35" s="8" t="n"/>
       <c r="AD35" s="8" t="n"/>
       <c r="AE35" s="8" t="n"/>
-      <c r="AF35" s="8" t="n"/>
-      <c r="AG35" s="8" t="n"/>
+      <c r="AF35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AG35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AH35" s="8" t="n"/>
       <c r="AL35" s="8" t="n"/>
       <c r="AM35" s="8" t="n"/>
@@ -8990,7 +8998,11 @@
       <c r="AC24" s="8" t="n"/>
       <c r="AD24" s="8" t="n"/>
       <c r="AE24" s="8" t="n"/>
-      <c r="AF24" s="8" t="n"/>
+      <c r="AF24" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AG24" s="8" t="n"/>
       <c r="AH24" s="8" t="n"/>
       <c r="AL24" s="8" t="n"/>
@@ -9939,8 +9951,16 @@
       <c r="AC43" s="8" t="n"/>
       <c r="AD43" s="8" t="n"/>
       <c r="AE43" s="8" t="n"/>
-      <c r="AF43" s="8" t="n"/>
-      <c r="AG43" s="8" t="n"/>
+      <c r="AF43" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="AG43" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AH43" s="8" t="n"/>
       <c r="AL43" s="8" t="n"/>
       <c r="AM43" s="8" t="n"/>
@@ -13109,7 +13129,11 @@
       <c r="AD36" s="8" t="n"/>
       <c r="AE36" s="8" t="n"/>
       <c r="AF36" s="8" t="n"/>
-      <c r="AG36" s="8" t="n"/>
+      <c r="AG36" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AH36" s="8" t="n"/>
       <c r="AL36" s="8" t="n"/>
       <c r="AM36" s="8" t="n"/>

</xml_diff>